<commit_message>
explannatory note updated 1
</commit_message>
<xml_diff>
--- a/statistcial power/Power_MDE_CKDev_Benin_summary.xlsx
+++ b/statistcial power/Power_MDE_CKDev_Benin_summary.xlsx
@@ -1,14 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RONALDO\CKDEV\GENDER NORMS\statistcial power\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC2417A-4151-499A-A58D-7316D948EBFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -225,8 +232,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -258,20 +265,351 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D63"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="64.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7265625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>5</v>
       </c>
@@ -282,12 +620,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="C3">
         <v>33</v>
@@ -296,12 +634,12 @@
         <v>1980</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C4">
         <v>52</v>
@@ -310,12 +648,12 @@
         <v>3120</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="C5">
         <v>70</v>
@@ -324,12 +662,12 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C6">
         <v>89</v>
@@ -338,12 +676,12 @@
         <v>5340</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>14</v>
       </c>
@@ -351,7 +689,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -362,7 +700,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -373,7 +711,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -384,7 +722,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -395,7 +733,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -406,12 +744,12 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>21</v>
       </c>
@@ -422,12 +760,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
       <c r="B18">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="C18">
         <v>0.16012373652001832</v>
@@ -436,12 +774,12 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
       <c r="B19">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C19">
         <v>0.20202493570966987</v>
@@ -450,12 +788,12 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
       <c r="B20">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="C20">
         <v>0.23661897282310276</v>
@@ -464,12 +802,12 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
       <c r="B21">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C21">
         <v>0.26676394424888877</v>
@@ -478,12 +816,12 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>37</v>
       </c>
@@ -494,26 +832,26 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>25</v>
       </c>
       <c r="B25">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="C25">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="D25">
         <v>57</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="C26">
         <v>0.25</v>
@@ -522,40 +860,40 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>27</v>
       </c>
       <c r="B27">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="C27">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="D27">
         <v>15</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>28</v>
       </c>
       <c r="B28">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C28">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="D28">
         <v>91</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>29</v>
       </c>
       <c r="B29">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C29">
         <v>0.25</v>
@@ -564,40 +902,40 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C30">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="D30">
         <v>23</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>31</v>
       </c>
       <c r="B31">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="C31">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="D31">
         <v>125</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="C32">
         <v>0.25</v>
@@ -606,40 +944,40 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="C33">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="D33">
         <v>32</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>34</v>
       </c>
       <c r="B34">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C34">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="D34">
         <v>159</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>35</v>
       </c>
       <c r="B35">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C35">
         <v>0.25</v>
@@ -648,26 +986,26 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>36</v>
       </c>
       <c r="B36">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C36">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="D36">
         <v>40</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
         <v>46</v>
       </c>
@@ -678,7 +1016,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -692,12 +1030,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>42</v>
       </c>
       <c r="B41">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C41">
         <v>0.19165768229748981</v>
@@ -706,12 +1044,12 @@
         <v>0.94868329805051377</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>43</v>
       </c>
       <c r="B42">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C42">
         <v>0.18069659575873537</v>
@@ -720,12 +1058,12 @@
         <v>0.89442719099991586</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>44</v>
       </c>
       <c r="B43">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="C43">
         <v>0.16902618807140221</v>
@@ -734,12 +1072,12 @@
         <v>0.83666002653407556</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>45</v>
       </c>
       <c r="B44">
-        <v>0.40000000000000002</v>
+        <v>0.4</v>
       </c>
       <c r="C44">
         <v>0.15648784230443843</v>
@@ -748,12 +1086,12 @@
         <v>0.7745966692414834</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>54</v>
       </c>
@@ -764,12 +1102,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>50</v>
       </c>
       <c r="B48">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="C48">
         <v>28.5</v>
@@ -778,12 +1116,12 @@
         <v>0.20324810492191164</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>51</v>
       </c>
       <c r="B49">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C49">
         <v>27</v>
@@ -792,12 +1130,12 @@
         <v>0.2045986055257295</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>52</v>
       </c>
       <c r="B50">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="C50">
         <v>25.5</v>
@@ -806,12 +1144,12 @@
         <v>0.20609751644734908</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>53</v>
       </c>
       <c r="B51">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C51">
         <v>24</v>
@@ -820,12 +1158,12 @@
         <v>0.20777086610324871</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>61</v>
       </c>
@@ -836,12 +1174,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>58</v>
       </c>
       <c r="B55">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="C55">
         <v>3000</v>
@@ -850,12 +1188,12 @@
         <v>0.82963049486309048</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>59</v>
       </c>
       <c r="B56">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="C56">
         <v>3000</v>
@@ -864,12 +1202,12 @@
         <v>0.99099180265622355</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>60</v>
       </c>
       <c r="B57">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C57">
         <v>3000</v>
@@ -878,12 +1216,12 @@
         <v>0.99992190980991225</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>65</v>
       </c>
@@ -891,7 +1229,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>66</v>
       </c>
@@ -899,7 +1237,7 @@
         <v>0.20200000000000001</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -907,7 +1245,7 @@
         <v>0.28599999999999998</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>68</v>
       </c>
@@ -916,5 +1254,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>